<commit_message>
All Animals Nuzzle Fork by [ETF] 번역 갱신
All Animals Nuzzle Fork by [ETF] - 3561546187
</commit_message>
<xml_diff>
--- a/Data/All Animals Nuzzle Fork by [ETF] - 3561546187/1.6/All Animals Nuzzle Fork by [ETF] - 3561546187.xlsx
+++ b/Data/All Animals Nuzzle Fork by [ETF] - 3561546187/1.6/All Animals Nuzzle Fork by [ETF] - 3561546187.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zilrt\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zilrt\Documents\Codex\2026-07-24\new-chat\outputs\translated_workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B194D8-85B5-4060-A054-FC62F48B0BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A423D4-563A-4DEA-A8CD-5320050F7EC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="170">
   <si>
     <t>Class+Node [(Identifier (Key)]</t>
   </si>
@@ -52,13 +52,7 @@
     <t>All Animals Nuzzle Settings</t>
   </si>
   <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Subtitle</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Subtitle</t>
-  </si>
-  <si>
-    <t>Auto-add Comfort to animals that can nuzzle so they cuddle more and boost colony vibes.</t>
+    <t>모든 동물 애교 설정</t>
   </si>
   <si>
     <t>Keyed+AllAnimalsNuzzle_UI_Subtitle_Comfort</t>
@@ -70,6 +64,9 @@
     <t>Auto-add Comfort to eligible animals (requires Odyssey to exist). Toggle to let animals learn cozy behavior.</t>
   </si>
   <si>
+    <t>대상 동물에게 '위로' 훈련을 자동으로 추가합니다(오디세이 DLC 필요). 동물이 다정한 행동을 배울 수 있도록 설정합니다.</t>
+  </si>
+  <si>
     <t>Keyed+AllAnimalsNuzzle_UI_Subtitle_Nuzzled</t>
   </si>
   <si>
@@ -79,6 +76,9 @@
     <t>Tweak the vanilla Nuzzled thought: duration, stacking, and per-stage mood boosts.</t>
   </si>
   <si>
+    <t>바닐라 '애교 받음' 생각의 지속 시간, 중첩, 단계별 기분 보너스를 조정합니다.</t>
+  </si>
+  <si>
     <t>Keyed+AllAnimalsNuzzle_UI_Tab_Comfort</t>
   </si>
   <si>
@@ -88,6 +88,9 @@
     <t>Comfort</t>
   </si>
   <si>
+    <t>위로</t>
+  </si>
+  <si>
     <t>Keyed+AllAnimalsNuzzle_UI_Tab_Nuzzled</t>
   </si>
   <si>
@@ -97,6 +100,9 @@
     <t>Nuzzled</t>
   </si>
   <si>
+    <t>애교 받음</t>
+  </si>
+  <si>
     <t>Keyed+AllAnimalsNuzzle_UI_OdysseyMissing</t>
   </si>
   <si>
@@ -106,6 +112,9 @@
     <t>Odyssey DLC not detected | Comfort option requires Odyssey to exist.</t>
   </si>
   <si>
+    <t>오디세이 DLC를 찾지 못했습니다 | '위로' 옵션을 사용하려면 오디세이 DLC가 필요합니다.</t>
+  </si>
+  <si>
     <t>Keyed+AllAnimalsNuzzle_UI_ComfortMissing</t>
   </si>
   <si>
@@ -115,6 +124,9 @@
     <t>The Comfort training is not present in your defs, so this option cannot be used.</t>
   </si>
   <si>
+    <t>현재 Def에 '위로' 훈련이 존재하지 않아 이 옵션을 사용할 수 없습니다.</t>
+  </si>
+  <si>
     <t>Keyed+AllAnimalsNuzzle_UI_Enable_Label</t>
   </si>
   <si>
@@ -124,272 +136,21 @@
     <t>Auto-add Comfort to nuzzling animals</t>
   </si>
   <si>
+    <t>애교를 부리는 동물에게 '위로' 자동 추가</t>
+  </si>
+  <si>
     <t>Keyed+AllAnimalsNuzzle_UI_Enable_Tooltip_Long</t>
   </si>
   <si>
     <t>AllAnimalsNuzzle_UI_Enable_Tooltip_Long</t>
   </si>
   <si>
-    <t xml:space="preserve">
-When enabled, the mod will add the Comfort trainable to animals that can nuzzle.
-What it does:
-- Leaves animals that already have Comfort alone.
-- Prevents duplicates.
-- If an animal had no &lt;specialTrainables/&gt;, the mod will create one and add Comfort.
-Turning it off will attempt to remove only the entries this mod added and restore original state where possible.
-  </t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_EnableLogging_Label</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_EnableLogging_Label</t>
-  </si>
-  <si>
-    <t>Show on-screen action messages</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_EnableLogging_Tooltip</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_EnableLogging_Tooltip</t>
-  </si>
-  <si>
-    <t>When enabled, the mod shows short on-screen messages when it adds or reverts Comfort. Useful for debugging.</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_TrackedHeading</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_TrackedHeading</t>
-  </si>
-  <si>
-    <t>Tracked changes: (What this mod changed)</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_None</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_None</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Message_Enabled</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Message_Enabled</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle: Comfort trainables added where appropriate.</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Message_Disabled</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Message_Disabled</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle: Previously added Comfort trainables removed where possible.</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_Method_CreatedList</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_Method_CreatedList</t>
-  </si>
-  <si>
-    <t>Created trainable list and added Comfort</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_Method_AddedExisting</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_Method_AddedExisting</t>
-  </si>
-  <si>
-    <t>Added Comfort to existing trainable list</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_Method_Unknown</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_Method_Unknown</t>
-  </si>
-  <si>
-    <t>Modified (unknown method)</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_ModName_Unknown</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_ModName_Unknown</t>
-  </si>
-  <si>
-    <t>Unknown mod</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Header</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_Header</t>
-  </si>
-  <si>
-    <t>Nuzzled Thought | Tweak Settings</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Duration_Label</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_Duration_Label</t>
-  </si>
-  <si>
-    <t>Duration (days)</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Duration_Tip</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_Duration_Tip</t>
-  </si>
-  <si>
-    <t>How long a nuzzle mood lasts on a pawn. Range between 0.1 through 60 days.</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_StackLimit_Label</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_StackLimit_Label</t>
-  </si>
-  <si>
-    <t>Max stacks</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_StackLimit_Tip</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_StackLimit_Tip</t>
-  </si>
-  <si>
-    <t>How many times the nuzzled mood can stack on a pawn. Range between 2 through 10.</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_StackedMultiplier_Label</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_StackedMultiplier_Label</t>
-  </si>
-  <si>
-    <t>Stack multiplier</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_StackedMultiplier_Tip</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_StackedMultiplier_Tip</t>
-  </si>
-  <si>
-    <t>Multiplier applied when multiple nuzzles stack. Range between 0.1 through 10.</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Stage0_Label</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_Stage0_Label</t>
-  </si>
-  <si>
-    <t>Stage 0 mood boost</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Stage0_Tip</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_Stage0_Tip</t>
-  </si>
-  <si>
-    <t>Base mood effect for stage 0. Range between 1 through 50.</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Stage1_Label</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_Stage1_Label</t>
-  </si>
-  <si>
-    <t>Stage 1 mood boost</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Stage1_Tip</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_Stage1_Tip</t>
-  </si>
-  <si>
-    <t>Base mood effect for stage 1. Range between 1 through 50.</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Reset_Button</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_Reset_Button</t>
-  </si>
-  <si>
-    <t>Reset to default</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Reset_Confirm</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_Reset_Confirm</t>
-  </si>
-  <si>
-    <t>Reset all Nuzzled settings to vanilla defaults? This cannot be undone except by reconfiguring the sliders.</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Reset_Done</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_UI_Nuzzled_Reset_Done</t>
-  </si>
-  <si>
-    <t>Nuzzled settings reset to vanilla defaults.</t>
-  </si>
-  <si>
-    <t>Keyed+AllAnimalsNuzzle_Debug_Cleared</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle_Debug_Cleared</t>
-  </si>
-  <si>
-    <t>AllAnimalsNuzzle: tracked modifications cleared.</t>
-  </si>
-  <si>
-    <t>모든 동물 애교 설정</t>
-  </si>
-  <si>
-    <t>애교를 부릴 수 있는 동물에게 '위로' 훈련을 자동으로 추가하여 더 자주 애교를 부리고 정착지 분위기를 북돋습니다.</t>
-  </si>
-  <si>
-    <t>대상 동물에게 '위로' 훈련을 자동으로 추가합니다(오디세이 DLC 필요). 동물이 다정한 행동을 배울 수 있도록 설정합니다.</t>
-  </si>
-  <si>
-    <t>바닐라 '애교 받음' 생각의 지속 시간, 중첩, 단계별 기분 보너스를 조정합니다.</t>
-  </si>
-  <si>
-    <t>위로</t>
-  </si>
-  <si>
-    <t>애교 받음</t>
-  </si>
-  <si>
-    <t>오디세이 DLC를 찾지 못했습니다 | '위로' 옵션을 사용하려면 오디세이 DLC가 필요합니다.</t>
-  </si>
-  <si>
-    <t>현재 Def에 '위로' 훈련이 존재하지 않아 이 옵션을 사용할 수 없습니다.</t>
-  </si>
-  <si>
-    <t>애교를 부리는 동물에게 '위로' 자동 추가</t>
+    <t>When enabled, the mod will add the Comfort trainable to animals that can nuzzle.
+    What it does:
+    - Leaves animals that already have Comfort alone.
+    - Prevents duplicates.
+    - If an animal had no &lt;specialTrainables/&gt;, the mod will create one and add Comfort.
+    Turning it off will attempt to remove only the entries this mod added and restore original state where possible.</t>
   </si>
   <si>
     <t>활성화하면 이 모드는 애교를 부릴 수 있는 동물에게 '위로' 훈련 항목을 추가합니다.
@@ -400,79 +161,385 @@
 비활성화하면 이 모드가 추가한 항목만 제거하고, 가능한 경우 원래 상태로 복원합니다.</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_EnableLogging_Label</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_EnableLogging_Label</t>
+  </si>
+  <si>
+    <t>Show on-screen action messages</t>
+  </si>
+  <si>
     <t>화면에 작업 메시지 표시</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_EnableLogging_Tooltip</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_EnableLogging_Tooltip</t>
+  </si>
+  <si>
+    <t>When enabled, the mod shows short on-screen messages when it adds or reverts Comfort. Useful for debugging.</t>
+  </si>
+  <si>
     <t>활성화하면 모드가 '위로'를 추가하거나 되돌릴 때 화면에 짧은 메시지를 표시합니다. 디버깅에 유용합니다.</t>
   </si>
   <si>
-    <t>추적된 변경 사항: (이 모드가 변경한 내용)</t>
+    <t>Keyed+AllAnimalsNuzzle_UI_TrackedHeading</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_TrackedHeading</t>
+  </si>
+  <si>
+    <t>Tracked Changes</t>
+  </si>
+  <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_None</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_None</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
   <si>
     <t>없음</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_ExpandAll</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_ExpandAll</t>
+  </si>
+  <si>
+    <t>Expand All</t>
+  </si>
+  <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_CollapseAll</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_CollapseAll</t>
+  </si>
+  <si>
+    <t>Collapse All</t>
+  </si>
+  <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Filter</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Filter</t>
+  </si>
+  <si>
+    <t>Filter:</t>
+  </si>
+  <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Clear</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Clear</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_NoTrackedChanges</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_NoTrackedChanges</t>
+  </si>
+  <si>
+    <t>No tracked def modifications match your filter.</t>
+  </si>
+  <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Show</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Show</t>
+  </si>
+  <si>
+    <t>Show</t>
+  </si>
+  <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Hide</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Hide</t>
+  </si>
+  <si>
+    <t>Hide</t>
+  </si>
+  <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Message_Enabled</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Message_Enabled</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle: Comfort trainables added where appropriate.</t>
+  </si>
+  <si>
     <t>AllAnimalsNuzzle: 해당하는 동물에게 '위로' 훈련 항목을 추가했습니다.</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Message_Disabled</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Message_Disabled</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle: Previously added Comfort trainables removed where possible.</t>
+  </si>
+  <si>
     <t>AllAnimalsNuzzle: 이전에 추가한 '위로' 훈련 항목을 가능한 범위에서 제거했습니다.</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_Method_CreatedList</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_Method_CreatedList</t>
+  </si>
+  <si>
+    <t>Created trainable list and added Comfort</t>
+  </si>
+  <si>
     <t>훈련 항목 목록을 생성하고 '위로'를 추가함</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_Method_AddedExisting</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_Method_AddedExisting</t>
+  </si>
+  <si>
+    <t>Added Comfort to existing trainable list</t>
+  </si>
+  <si>
     <t>기존 훈련 항목 목록에 '위로'를 추가함</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_Method_Unknown</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_Method_Unknown</t>
+  </si>
+  <si>
+    <t>Modified (unknown method)</t>
+  </si>
+  <si>
     <t>수정됨(알 수 없는 방식)</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_ModName_Unknown</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_ModName_Unknown</t>
+  </si>
+  <si>
+    <t>Unknown mod</t>
+  </si>
+  <si>
     <t>알 수 없는 모드</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Header</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_Header</t>
+  </si>
+  <si>
+    <t>Nuzzled Thought | Tweak Settings</t>
+  </si>
+  <si>
     <t>애교 받음 생각 | 설정 조정</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Duration_Label</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_Duration_Label</t>
+  </si>
+  <si>
+    <t>Duration (days)</t>
+  </si>
+  <si>
     <t>지속 시간(일)</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Duration_Tip</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_Duration_Tip</t>
+  </si>
+  <si>
+    <t>How long a nuzzle mood lasts on a pawn. Range between 0.1 through 60 days.</t>
+  </si>
+  <si>
     <t>'애교 받음' 기분이 지속되는 시간입니다. 0.1일에서 60일까지 설정할 수 있습니다.</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_StackLimit_Label</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_StackLimit_Label</t>
+  </si>
+  <si>
+    <t>Max stacks</t>
+  </si>
+  <si>
     <t>최대 중첩 수</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_StackLimit_Tip</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_StackLimit_Tip</t>
+  </si>
+  <si>
+    <t>How many times the nuzzled mood can stack on a pawn. Range between 2 through 10.</t>
+  </si>
+  <si>
     <t>'애교 받음' 기분이 한 대상에게 중첩될 수 있는 횟수입니다. 2회에서 10회까지 설정할 수 있습니다.</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_StackedMultiplier_Label</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_StackedMultiplier_Label</t>
+  </si>
+  <si>
+    <t>Stack multiplier</t>
+  </si>
+  <si>
     <t>중첩 배율</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_StackedMultiplier_Tip</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_StackedMultiplier_Tip</t>
+  </si>
+  <si>
+    <t>Multiplier applied when multiple nuzzles stack. Range between 0.1 through 10.</t>
+  </si>
+  <si>
     <t>애교가 여러 번 중첩될 때 적용되는 배율입니다. 0.1배에서 10배까지 설정할 수 있습니다.</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Stage0_Label</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_Stage0_Label</t>
+  </si>
+  <si>
+    <t>Stage 0 mood boost</t>
+  </si>
+  <si>
     <t>0단계 기분 보너스</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Stage0_Tip</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_Stage0_Tip</t>
+  </si>
+  <si>
+    <t>Base mood effect for stage 0. Range between 1 through 50.</t>
+  </si>
+  <si>
     <t>0단계의 기본 기분 효과입니다. 1에서 50까지 설정할 수 있습니다.</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Stage1_Label</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_Stage1_Label</t>
+  </si>
+  <si>
+    <t>Stage 1 mood boost</t>
+  </si>
+  <si>
     <t>1단계 기분 보너스</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Stage1_Tip</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_Stage1_Tip</t>
+  </si>
+  <si>
+    <t>Base mood effect for stage 1. Range between 1 through 50.</t>
+  </si>
+  <si>
     <t>1단계의 기본 기분 효과입니다. 1에서 50까지 설정할 수 있습니다.</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Reset_Button</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_Reset_Button</t>
+  </si>
+  <si>
+    <t>Reset to default</t>
+  </si>
+  <si>
     <t>기본값으로 초기화</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Reset_Confirm</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_Reset_Confirm</t>
+  </si>
+  <si>
+    <t>Reset all Nuzzled settings to vanilla defaults? This cannot be undone except by reconfiguring the sliders.</t>
+  </si>
+  <si>
     <t>모든 '애교 받음' 설정을 바닐라 기본값으로 초기화하시겠습니까? 슬라이더를 다시 설정하는 것 외에는 되돌릴 수 없습니다.</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_UI_Nuzzled_Reset_Done</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_UI_Nuzzled_Reset_Done</t>
+  </si>
+  <si>
+    <t>Nuzzled settings reset to vanilla defaults.</t>
+  </si>
+  <si>
     <t>'애교 받음' 설정을 바닐라 기본값으로 초기화했습니다.</t>
   </si>
   <si>
+    <t>Keyed+AllAnimalsNuzzle_Debug_Cleared</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle_Debug_Cleared</t>
+  </si>
+  <si>
+    <t>AllAnimalsNuzzle: tracked modifications cleared.</t>
+  </si>
+  <si>
     <t>AllAnimalsNuzzle: 추적된 변경 사항을 지웠습니다.</t>
+  </si>
+  <si>
+    <t>추적된 변경 사항</t>
+  </si>
+  <si>
+    <t>모두 펼치기</t>
+  </si>
+  <si>
+    <t>모두 접기</t>
+  </si>
+  <si>
+    <t>필터:</t>
+  </si>
+  <si>
+    <t>필터와 일치하는 추적된 Def 수정 사항이 없습니다.</t>
+  </si>
+  <si>
+    <t>표시</t>
+  </si>
+  <si>
+    <t>숨기기</t>
   </si>
 </sst>
 </file>
@@ -519,10 +586,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -541,7 +609,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -583,9 +651,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -598,12 +666,52 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="dk1"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="accent1"/>
-        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525">
@@ -661,7 +769,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -687,7 +795,7 @@
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -716,20 +824,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="40.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="56.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="68.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="37.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="67.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="72.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="9.140625" style="1" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -749,7 +857,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -762,586 +870,689 @@
       <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="G13"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>126</v>
+        <v>63</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>127</v>
+        <v>66</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>128</v>
+        <v>69</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>129</v>
+        <v>72</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>130</v>
+        <v>75</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>131</v>
+        <v>78</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>132</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>133</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>135</v>
+        <v>94</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>136</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>137</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>138</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>139</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>140</v>
+        <v>113</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>141</v>
+        <v>117</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>142</v>
+        <v>121</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>143</v>
+        <v>125</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>144</v>
+        <v>129</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>145</v>
+        <v>133</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>109</v>
+        <v>135</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>110</v>
+        <v>136</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F36" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>146</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>